<commit_message>
scan: seg5 2026-08-12 18:02 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq6_2026-08-12.xlsx
+++ b/output/full_scan/batch_seq6_2026-08-12.xlsx
@@ -633,21 +633,21 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>6213</v>
+        <v>6279</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>聯茂</t>
+          <t>胡連</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
         <v/>
       </c>
       <c r="D4" s="2" t="n">
-        <v>802.9738799416245</v>
+        <v>775.8003676364793</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>464</v>
+        <v>130.5</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -658,16 +658,16 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>72.05012262411302</v>
+        <v>71.71218241200081</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>21.33862737858883</v>
+        <v>20.8750072235637</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>0.3973879941624552</v>
+        <v>1.180036763647935</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>0</v>
@@ -676,31 +676,31 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>18.23536009771396</v>
+        <v>1.88324459592807</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, foreign_buy_3d, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>6279</v>
+        <v>6183</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>胡連</t>
+          <t>關貿</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
         <v/>
       </c>
       <c r="D5" s="2" t="n">
-        <v>775.8003676364793</v>
+        <v>731.8825377555555</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>130.5</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -711,16 +711,16 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>71.71218241200081</v>
+        <v>63.65774546811014</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>20.8750072235637</v>
+        <v>28.42012880117692</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>1.180036763647935</v>
+        <v>1.600335806818372</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>0</v>
@@ -729,31 +729,31 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>1.88324459592807</v>
+        <v>0.2044787413374985</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, foreign_buy_3d, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>6426</v>
+        <v>6206</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>統新</t>
+          <t>飛捷</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
         <v/>
       </c>
       <c r="D6" s="2" t="n">
-        <v>734.4304792857854</v>
+        <v>681.8421829244294</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>222</v>
+        <v>146</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -764,13 +764,13 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>66.2965654031747</v>
+        <v>58.04295084549359</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>25.46364121108727</v>
+        <v>24.42562205314122</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>0.7262887659606406</v>
+        <v>0.6456812908259706</v>
       </c>
       <c r="K6" s="2" t="n">
         <v>0</v>
@@ -782,31 +782,31 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>9.286858591947439</v>
+        <v>2.283188567167719</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>6183</v>
+        <v>6446</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>關貿</t>
+          <t>藥華藥</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>731.8825377555555</v>
+        <v>671.7016960211546</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>94.40000000000001</v>
+        <v>1440</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -817,13 +817,13 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>63.65774546811014</v>
+        <v>63.61728612548056</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>28.42012880117692</v>
+        <v>27.35698828431211</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>1.600335806818372</v>
+        <v>1.7218746142186</v>
       </c>
       <c r="K7" s="2" t="n">
         <v>0</v>
@@ -835,31 +835,31 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.2044787413374985</v>
+        <v>28.10479582509499</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, bb_squeeze_breakout, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>6206</v>
+        <v>6292</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>飛捷</t>
+          <t>迅德</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>681.8421829244294</v>
+        <v>669.9103574305414</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>146</v>
+        <v>66.3</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -870,13 +870,13 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>58.04295084549359</v>
+        <v>67.76947010214028</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>24.42562205314122</v>
+        <v>22.58778208965134</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>0.6456812908259706</v>
+        <v>7.698364578741617</v>
       </c>
       <c r="K8" s="2" t="n">
         <v>0</v>
@@ -888,31 +888,31 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>2.283188567167719</v>
+        <v>1.818148352826847</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, adx_trending, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>6446</v>
+        <v>6173</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>藥華藥</t>
+          <t>信昌電</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>671.7016960211546</v>
+        <v>614</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>1440</v>
+        <v>203.5</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -923,13 +923,13 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>63.61728612548056</v>
+        <v>53.16869881903645</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>27.35698828431211</v>
+        <v>31.0234502825572</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>1.7218746142186</v>
+        <v>5.093891790975618</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>0</v>
@@ -941,31 +941,31 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>28.10479582509499</v>
+        <v>6.385738221690421</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, bb_squeeze_breakout, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>6292</v>
+        <v>6217</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>迅德</t>
+          <t>中探針</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>669.9103574305414</v>
+        <v>610.6018155769365</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>66.3</v>
+        <v>154</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -976,16 +976,16 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>67.76947010214028</v>
+        <v>42.80856712330261</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>22.58778208965134</v>
+        <v>24.42453444847061</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>7.698364578741617</v>
+        <v>0.2864235519521297</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L10" s="2" t="n">
         <v>0</v>
@@ -994,31 +994,31 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>1.818148352826847</v>
+        <v>6.233716883481648</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, adx_trending, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>6173</v>
+        <v>6223</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>信昌電</t>
+          <t>旺矽</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
         <v/>
       </c>
       <c r="D11" s="2" t="n">
-        <v>614</v>
+        <v>601.7983368931973</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>203.5</v>
+        <v>6600</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -1029,49 +1029,49 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>53.16869881903645</v>
+        <v>58.4711575727979</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>31.0234502825572</v>
+        <v>14.84701981456528</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>5.093891790975618</v>
+        <v>0.6720354601043514</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M11" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>6.385738221690421</v>
+        <v>123.0915105316088</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, obv_uptrend, invest_trust_buy_2d, cci_momentum</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>6223</v>
+        <v>6416</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>旺矽</t>
+          <t>瑞祺電通</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>601.7983368931973</v>
+        <v>578.2443216025605</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>6600</v>
+        <v>100</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -1082,49 +1082,49 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>58.4711575727979</v>
+        <v>55.76187137709232</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>14.84701981456528</v>
+        <v>20.5751291680424</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>0.6720354601043514</v>
+        <v>0.6837426354283923</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M12" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>123.0915105316088</v>
+        <v>0.159011541872748</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, obv_uptrend, invest_trust_buy_2d, cci_momentum</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>6416</v>
+        <v>6414</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>瑞祺電通</t>
+          <t>樺漢</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>578.2443216025605</v>
+        <v>572.6925605931161</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>100</v>
+        <v>455.5</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -1135,13 +1135,13 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>55.76187137709232</v>
+        <v>55.45419913227837</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>20.5751291680424</v>
+        <v>20.59797859383072</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>0.6837426354283923</v>
+        <v>0.3599746686654043</v>
       </c>
       <c r="K13" s="2" t="n">
         <v>0</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.159011541872748</v>
+        <v>-0.7890241319810407</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1163,21 +1163,21 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>6414</v>
+        <v>6442</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>樺漢</t>
+          <t>光聖</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>572.6925605931161</v>
+        <v>566.1785100163833</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>455.5</v>
+        <v>1595</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -1188,13 +1188,13 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>55.45419913227837</v>
+        <v>58.68867130380801</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>20.59797859383072</v>
+        <v>21.39846210885802</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>0.3599746686654043</v>
+        <v>1.212931608579403</v>
       </c>
       <c r="K14" s="2" t="n">
         <v>0</v>
@@ -1206,31 +1206,31 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>-0.7890241319810407</v>
+        <v>52.694936706427</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
+          <t>rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>6442</v>
+        <v>6472</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>光聖</t>
+          <t>保瑞</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v/>
       </c>
       <c r="D15" s="2" t="n">
-        <v>566.1785100163833</v>
+        <v>566.1763634879791</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>1595</v>
+        <v>424</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1241,13 +1241,13 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>58.68867130380801</v>
+        <v>56.1239449390891</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>21.39846210885802</v>
+        <v>22.80703223942334</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>1.212931608579403</v>
+        <v>0.8479480364742736</v>
       </c>
       <c r="K15" s="2" t="n">
         <v>0</v>
@@ -1259,31 +1259,31 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>52.694936706427</v>
+        <v>3.878017969196611</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>6472</v>
+        <v>6419</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>保瑞</t>
+          <t>京晨科</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>566.1763634879791</v>
+        <v>563.9134801640168</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>424</v>
+        <v>153</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -1294,16 +1294,16 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>56.1239449390891</v>
+        <v>59.433366381644</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>22.80703223942334</v>
+        <v>14.48903112977805</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>0.8479480364742736</v>
+        <v>1.662502658517891</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>0</v>
@@ -1312,31 +1312,31 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>3.878017969196611</v>
+        <v>3.032913967159091</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, obv_uptrend, breakout_volume_confirm, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>6419</v>
+        <v>6432</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>京晨科</t>
+          <t>今展科</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
         <v/>
       </c>
       <c r="D17" s="2" t="n">
-        <v>563.9134801640168</v>
+        <v>554.9860077309886</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>153</v>
+        <v>74</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1347,16 +1347,16 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>59.433366381644</v>
+        <v>52.64084730703163</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>14.48903112977805</v>
+        <v>11.0096014298274</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>1.662502658517891</v>
+        <v>0.7504299600880644</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L17" s="2" t="n">
         <v>0</v>
@@ -1365,31 +1365,31 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>3.032913967159091</v>
+        <v>0.0511037697348957</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, obv_uptrend, breakout_volume_confirm, mfi_strong</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>6432</v>
+        <v>6216</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>今展科</t>
+          <t>居易</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>554.9860077309886</v>
+        <v>551.5380026398415</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>74</v>
+        <v>22.8</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1400,13 +1400,13 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>52.64084730703163</v>
+        <v>61.87466645769963</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>11.0096014298274</v>
+        <v>14.17471811391077</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>0.7504299600880644</v>
+        <v>1.618951656291325</v>
       </c>
       <c r="K18" s="2" t="n">
         <v>0</v>
@@ -1418,31 +1418,31 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>0.0511037697348957</v>
+        <v>0.1231609957363036</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, dealer_buy_3d, mfi_strong</t>
+          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, obv_uptrend, bb_squeeze_breakout, breakout_volume_confirm</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>6216</v>
+        <v>6227</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>居易</t>
+          <t>茂綸</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>551.5380026398415</v>
+        <v>542.4350305370961</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>22.8</v>
+        <v>125.5</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1453,13 +1453,13 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>61.87466645769963</v>
+        <v>57.35372367186925</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>14.17471811391077</v>
+        <v>16.24650773323673</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>1.618951656291325</v>
+        <v>2.182143295615714</v>
       </c>
       <c r="K19" s="2" t="n">
         <v>0</v>
@@ -1471,31 +1471,31 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.1231609957363036</v>
+        <v>1.763240161441672</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, obv_uptrend, bb_squeeze_breakout, breakout_volume_confirm</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>6227</v>
+        <v>6241</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>茂綸</t>
+          <t>鑫永洋</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
         <v/>
       </c>
       <c r="D20" s="2" t="n">
-        <v>542.4350305370961</v>
+        <v>510.6743737008134</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>125.5</v>
+        <v>14.35</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1506,16 +1506,16 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>57.35372367186925</v>
+        <v>40.81004745249126</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>16.24650773323673</v>
+        <v>23.62519808028881</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>2.182143295615714</v>
+        <v>0.4821325726296193</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>0</v>
@@ -1524,31 +1524,31 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>1.763240161441672</v>
+        <v>-0.3517713050738112</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>6451</v>
+        <v>6474</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>訊芯-KY</t>
+          <t>華豫寧</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
         <v/>
       </c>
       <c r="D21" s="2" t="n">
-        <v>538.3948711419972</v>
+        <v>503.1587973640962</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>451</v>
+        <v>39.1</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1559,16 +1559,16 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>51.25061681796154</v>
+        <v>58.7209737517258</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>18.30058381248198</v>
+        <v>9.160002015182693</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>0.3174585377150971</v>
+        <v>1.200184708753876</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" s="2" t="n">
         <v>0</v>
@@ -1577,31 +1577,31 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>12.18525629364846</v>
+        <v>0.2107650134734091</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>6241</v>
+        <v>6215</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>鑫永洋</t>
+          <t>和椿</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>510.6743737008134</v>
+        <v>501.1293170238585</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>14.35</v>
+        <v>104.5</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1612,16 +1612,16 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>40.81004745249126</v>
+        <v>56.75745477048399</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>23.62519808028881</v>
+        <v>19.9722646624082</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>0.4821325726296193</v>
+        <v>1.557620710594771</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L22" s="2" t="n">
         <v>0</v>
@@ -1630,31 +1630,31 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>-0.3517713050738112</v>
+        <v>2.103842171684908</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, above_ichimoku_cloud</t>
+          <t>volume_break, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>6474</v>
+        <v>6214</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>華豫寧</t>
+          <t>精誠</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>503.1587973640962</v>
+        <v>500.7449223661498</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>39.1</v>
+        <v>142.5</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -1665,16 +1665,16 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>58.7209737517258</v>
+        <v>49.32221572399222</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>9.160002015182693</v>
+        <v>12.88807517690204</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>1.200184708753876</v>
+        <v>0.3250436227196002</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
         <v>0</v>
@@ -1683,31 +1683,31 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.2107650134734091</v>
+        <v>-0.6578902815666918</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>6215</v>
+        <v>6435</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>和椿</t>
+          <t>大中</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>501.1293170238585</v>
+        <v>500.1695121551197</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>104.5</v>
+        <v>261.5</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1718,16 +1718,16 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>56.75745477048399</v>
+        <v>45.8375414530556</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>19.9722646624082</v>
+        <v>28.66490800318767</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>1.557620710594771</v>
+        <v>0.6656040097256752</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>0</v>
@@ -1736,31 +1736,31 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>2.103842171684908</v>
+        <v>2.507828533119358</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>6214</v>
+        <v>6271</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>精誠</t>
+          <t>同欣電</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>500.7449223661498</v>
+        <v>497.9058360127173</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>142.5</v>
+        <v>198</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1771,13 +1771,13 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>49.32221572399222</v>
+        <v>49.45612857916011</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>12.88807517690204</v>
+        <v>20.77988378650916</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>0.3250436227196002</v>
+        <v>0.6602310246239508</v>
       </c>
       <c r="K25" s="2" t="n">
         <v>0</v>
@@ -1789,31 +1789,31 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-0.6578902815666918</v>
+        <v>4.505145439186419</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>6435</v>
+        <v>6275</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>大中</t>
+          <t>元山</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>500.1695121551197</v>
+        <v>497.2731825235641</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>261.5</v>
+        <v>44.6</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1824,16 +1824,16 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>45.8375414530556</v>
+        <v>49.48573511372874</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>28.66490800318767</v>
+        <v>24.21292980768262</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>0.6656040097256752</v>
+        <v>1.911519286352609</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L26" s="2" t="n">
         <v>0</v>
@@ -1842,31 +1842,31 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>2.507828533119358</v>
+        <v>0.427874758093272</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>6271</v>
+        <v>6245</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>同欣電</t>
+          <t>立端</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>497.9058360127173</v>
+        <v>495.2599277520185</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>198</v>
+        <v>88</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1877,16 +1877,16 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>49.45612857916011</v>
+        <v>62.67191244494753</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>20.77988378650916</v>
+        <v>15.00401131930726</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.6602310246239508</v>
+        <v>0.7848851871245506</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L27" s="2" t="n">
         <v>0</v>
@@ -1895,31 +1895,31 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>4.505145439186419</v>
+        <v>1.196816494855589</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>6275</v>
+        <v>6284</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>元山</t>
+          <t>佳邦</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>497.2731825235641</v>
+        <v>495.1527216793516</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>44.6</v>
+        <v>79.3</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1930,16 +1930,16 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>49.48573511372874</v>
+        <v>46.77236058247347</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>24.21292980768262</v>
+        <v>26.49988634004748</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>1.911519286352609</v>
+        <v>0.6694108853584463</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L28" s="2" t="n">
         <v>0</v>
@@ -1948,31 +1948,31 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.427874758093272</v>
+        <v>1.177327618986959</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>6245</v>
+        <v>6175</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>立端</t>
+          <t>立敦</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>495.2599277520185</v>
+        <v>484.929602263951</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>88</v>
+        <v>78.5</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,13 +1983,13 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>62.67191244494753</v>
+        <v>42.81141513557344</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>15.00401131930726</v>
+        <v>24.25431589411448</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>0.7848851871245506</v>
+        <v>0.4302503757199974</v>
       </c>
       <c r="K29" s="2" t="n">
         <v>1</v>
@@ -2001,31 +2001,31 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>1.196816494855589</v>
+        <v>0.7286056010057953</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>6284</v>
+        <v>6207</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>佳邦</t>
+          <t>雷科</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>495.1527216793516</v>
+        <v>481.1664982566279</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>79.3</v>
+        <v>111.5</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2036,13 +2036,13 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46.77236058247347</v>
+        <v>48.46273937646578</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>26.49988634004748</v>
+        <v>21.57549336510453</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>0.6694108853584463</v>
+        <v>0.9060534827941932</v>
       </c>
       <c r="K30" s="2" t="n">
         <v>1</v>
@@ -2054,31 +2054,31 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>1.177327618986959</v>
+        <v>1.311271994623251</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>6175</v>
+        <v>6423</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>立敦</t>
+          <t>億而得-創</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>484.929602263951</v>
+        <v>468.9870350167013</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>78.5</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2089,16 +2089,16 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>42.81141513557344</v>
+        <v>59.11163340968611</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>24.25431589411448</v>
+        <v>23.84029231794083</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.4302503757199974</v>
+        <v>0.575574697741415</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L31" s="2" t="n">
         <v>0</v>
@@ -2107,31 +2107,31 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.7286056010057953</v>
+        <v>1.998861775783007</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, dealer_buy_3d</t>
+          <t>rsi_strong, market_above_ma60, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>6207</v>
+        <v>6277</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>雷科</t>
+          <t>宏正</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>481.1664982566279</v>
+        <v>468.1855837319367</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>111.5</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,16 +2142,16 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>48.46273937646578</v>
+        <v>54.55881564207451</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>21.57549336510453</v>
+        <v>40.21101461668024</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0.9060534827941932</v>
+        <v>0.3823331718529587</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L32" s="2" t="n">
         <v>0</v>
@@ -2160,31 +2160,31 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>1.311271994623251</v>
+        <v>0.0438541854873035</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>6423</v>
+        <v>6204</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>億而得-創</t>
+          <t>艾華</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>468.9870350167013</v>
+        <v>460.5301586009954</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>81.09999999999999</v>
+        <v>85.5</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,16 +2195,16 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>59.11163340968611</v>
+        <v>54.87215863446699</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>23.84029231794083</v>
+        <v>28.64068332160533</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>0.575574697741415</v>
+        <v>1.262827535483691</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>0</v>
@@ -2213,31 +2213,31 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>1.998861775783007</v>
+        <v>2.836567919626379</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>6277</v>
+        <v>6218</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>宏正</t>
+          <t>豪勉</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>468.1855837319367</v>
+        <v>458.4188893796352</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>78.59999999999999</v>
+        <v>36.15</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2248,13 +2248,13 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>54.55881564207451</v>
+        <v>56.47559033857147</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>40.21101461668024</v>
+        <v>13.22414919935149</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>0.3823331718529587</v>
+        <v>2.284205768095775</v>
       </c>
       <c r="K34" s="2" t="n">
         <v>0</v>
@@ -2266,31 +2266,31 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.0438541854873035</v>
+        <v>0.5510804499995686</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>6204</v>
+        <v>6177</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>艾華</t>
+          <t>達麗</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>460.5301586009954</v>
+        <v>457.738150365368</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>85.5</v>
+        <v>47.7</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,16 +2301,16 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>54.87215863446699</v>
+        <v>52.7247068469344</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>28.64068332160533</v>
+        <v>27.04975270427772</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>1.262827535483691</v>
+        <v>1.058874845774771</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L35" s="2" t="n">
         <v>0</v>
@@ -2319,31 +2319,31 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>2.836567919626379</v>
+        <v>-0.0152050327342894</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>6218</v>
+        <v>6192</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>豪勉</t>
+          <t>巨路</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>458.4188893796352</v>
+        <v>457.2873679337393</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>36.15</v>
+        <v>120.5</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2354,13 +2354,13 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>56.47559033857147</v>
+        <v>59.36782520899812</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>13.22414919935149</v>
+        <v>25.49425602909804</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>2.284205768095775</v>
+        <v>1.102704144774383</v>
       </c>
       <c r="K36" s="2" t="n">
         <v>0</v>
@@ -2372,31 +2372,31 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>0.5510804499995686</v>
+        <v>1.202773362699608</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>6177</v>
+        <v>6274</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>達麗</t>
+          <t>台燿</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>457.738150365368</v>
+        <v>454.5924173780477</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>47.7</v>
+        <v>1600</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2407,13 +2407,13 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>52.7247068469344</v>
+        <v>59.70091078811382</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>27.04975270427772</v>
+        <v>16.41942089096488</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>1.058874845774771</v>
+        <v>0.3891128928594383</v>
       </c>
       <c r="K37" s="2" t="n">
         <v>0</v>
@@ -2425,31 +2425,31 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-0.0152050327342894</v>
+        <v>55.77620990790869</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>6192</v>
+        <v>6224</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>巨路</t>
+          <t>聚鼎</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>457.2873679337393</v>
+        <v>452.4069617705631</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>120.5</v>
+        <v>61.2</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2460,13 +2460,13 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>59.36782520899812</v>
+        <v>51.08849900209115</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>25.49425602909804</v>
+        <v>29.22230671159344</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>1.102704144774383</v>
+        <v>1.492379912380631</v>
       </c>
       <c r="K38" s="2" t="n">
         <v>0</v>
@@ -2478,31 +2478,31 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>1.202773362699608</v>
+        <v>1.509661775879946</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>6224</v>
+        <v>6191</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>聚鼎</t>
+          <t>精成科</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>452.4069617705631</v>
+        <v>447.5338903769803</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>61.2</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2513,13 +2513,13 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>51.08849900209115</v>
+        <v>46.34643372684511</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>29.22230671159344</v>
+        <v>30.79416751280549</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>1.492379912380631</v>
+        <v>0.5122135713279935</v>
       </c>
       <c r="K39" s="2" t="n">
         <v>0</v>
@@ -2531,31 +2531,31 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>1.509661775879946</v>
+        <v>0.7596909364932141</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>6191</v>
+        <v>6246</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>精成科</t>
+          <t>臺龍</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>447.5338903769803</v>
+        <v>446.5789651731137</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>87.09999999999999</v>
+        <v>13.35</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2566,16 +2566,16 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>46.34643372684511</v>
+        <v>50.05105480618104</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>30.79416751280549</v>
+        <v>26.22831861324728</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>0.5122135713279935</v>
+        <v>3.545000647124126</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L40" s="2" t="n">
         <v>0</v>
@@ -2584,31 +2584,31 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.7596909364932141</v>
+        <v>0.1117673909700633</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>6246</v>
+        <v>6269</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>臺龍</t>
+          <t>台郡</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>446.5789651731137</v>
+        <v>445.7276435842268</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>13.35</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2619,16 +2619,16 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>50.05105480618104</v>
+        <v>59.9104521754532</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>26.22831861324728</v>
+        <v>22.42294149089513</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>3.545000647124126</v>
+        <v>1.294095971468612</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L41" s="2" t="n">
         <v>0</v>
@@ -2637,31 +2637,31 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.1117673909700633</v>
+        <v>2.169845386300168</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>6269</v>
+        <v>6243</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>台郡</t>
+          <t>迅杰</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>445.7276435842268</v>
+        <v>444.7731607567517</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>66.90000000000001</v>
+        <v>44.55</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2672,13 +2672,13 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>59.9104521754532</v>
+        <v>48.00169324058536</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>22.42294149089513</v>
+        <v>21.3459098817867</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>1.294095971468612</v>
+        <v>0.1773090515354023</v>
       </c>
       <c r="K42" s="2" t="n">
         <v>0</v>
@@ -2690,31 +2690,31 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>2.169845386300168</v>
+        <v>-0.9548358842638494</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>6243</v>
+        <v>6163</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>迅杰</t>
+          <t>華電網</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>444.7731607567517</v>
+        <v>442.7968906294115</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>44.55</v>
+        <v>43.1</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2725,16 +2725,16 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>48.00169324058536</v>
+        <v>51.1135821924035</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>21.3459098817867</v>
+        <v>24.97403065340221</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.1773090515354023</v>
+        <v>0.7845036196931419</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L43" s="2" t="n">
         <v>0</v>
@@ -2743,31 +2743,31 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-0.9548358842638494</v>
+        <v>0.7643451430549173</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, cci_momentum</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>6163</v>
+        <v>6290</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>華電網</t>
+          <t>良維</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>442.7968906294115</v>
+        <v>441.4772301840677</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>43.1</v>
+        <v>218.5</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,16 +2778,16 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>51.1135821924035</v>
+        <v>41.10302311337608</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>24.97403065340221</v>
+        <v>36.13106072806133</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.7845036196931419</v>
+        <v>0.6035163729903129</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L44" s="2" t="n">
         <v>0</v>
@@ -2796,31 +2796,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.7643451430549173</v>
+        <v>2.675551292355465</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, cci_momentum</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>6290</v>
+        <v>6225</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>良維</t>
+          <t>天瀚</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>441.4772301840677</v>
+        <v>439.4819759606579</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>218.5</v>
+        <v>33.45</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,13 +2831,13 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>41.10302311337608</v>
+        <v>75.85492741633625</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>36.13106072806133</v>
+        <v>18.04260385340267</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>0.6035163729903129</v>
+        <v>0.5481975960657924</v>
       </c>
       <c r="K45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>2.675551292355465</v>
+        <v>0.8704943153711531</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6225</v>
+        <v>6261</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>天瀚</t>
+          <t>久元</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>439.4819759606579</v>
+        <v>436.7142656095471</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>33.45</v>
+        <v>79.2</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,16 +2884,16 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>75.85492741633625</v>
+        <v>42.38770913928385</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>18.04260385340267</v>
+        <v>33.08118207998002</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0.5481975960657924</v>
+        <v>0.6026194184084672</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.8704943153711531</v>
+        <v>0.8887775360010126</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>6261</v>
+        <v>6465</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>久元</t>
+          <t>威潤</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>436.7142656095471</v>
+        <v>434.1705023758108</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>79.2</v>
+        <v>47.5</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,16 +2937,16 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>42.38770913928385</v>
+        <v>37.16443438992344</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>33.08118207998002</v>
+        <v>17.25168231066607</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.6026194184084672</v>
+        <v>0.4612457197580284</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L47" s="2" t="n">
         <v>0</v>
@@ -2955,31 +2955,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.8887775360010126</v>
+        <v>0.1176494507744001</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>6465</v>
+        <v>6190</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>威潤</t>
+          <t>萬泰科</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>434.1705023758108</v>
+        <v>431.5010564422908</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>47.5</v>
+        <v>68.8</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,13 +2990,13 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>37.16443438992344</v>
+        <v>47.05627034549753</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>17.25168231066607</v>
+        <v>30.41596882464223</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.4612457197580284</v>
+        <v>0.8700589067430139</v>
       </c>
       <c r="K48" s="2" t="n">
         <v>1</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.1176494507744001</v>
+        <v>0.8044301408871055</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>6190</v>
+        <v>6236</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>萬泰科</t>
+          <t>中湛</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>431.5010564422908</v>
+        <v>429</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>68.8</v>
+        <v>15.35</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,16 +3043,16 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>47.05627034549753</v>
+        <v>76.04474913525762</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>30.41596882464223</v>
+        <v>8.017174027052567</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.8700589067430139</v>
+        <v>20</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.8044301408871055</v>
+        <v>1.053316519521084</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend</t>
+          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, obv_uptrend, breakout_volume_confirm, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>6236</v>
+        <v>6282</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>中湛</t>
+          <t>康舒</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>429</v>
+        <v>423.8125026962184</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>15.35</v>
+        <v>47.15</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,13 +3096,13 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>76.04474913525762</v>
+        <v>45.47295622217041</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>8.017174027052567</v>
+        <v>20.58247646586054</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>20</v>
+        <v>1.656058258311744</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>1.053316519521084</v>
+        <v>0.8094095698939294</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, obv_uptrend, breakout_volume_confirm, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>6282</v>
+        <v>6165</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>康舒</t>
+          <t>浪凡</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>423.8125026962184</v>
+        <v>422.9446024527382</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>47.15</v>
+        <v>49.6</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,13 +3149,13 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>45.47295622217041</v>
+        <v>50.75884989430282</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>20.58247646586054</v>
+        <v>14.61126007353877</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>1.656058258311744</v>
+        <v>0.4272497710122562</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.8094095698939294</v>
+        <v>0.1079741116639171</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>6165</v>
+        <v>6197</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>浪凡</t>
+          <t>佳必琪</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>422.9446024527382</v>
+        <v>416.46575512166</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>49.6</v>
+        <v>305.5</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,13 +3202,13 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>50.75884989430282</v>
+        <v>48.30651527988162</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>14.61126007353877</v>
+        <v>18.14262281634702</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.4272497710122562</v>
+        <v>0.5320092646604917</v>
       </c>
       <c r="K52" s="2" t="n">
         <v>0</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.1079741116639171</v>
+        <v>1.174972219069714</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3230,21 +3230,21 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>6197</v>
+        <v>6202</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>佳必琪</t>
+          <t>盛群</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>416.46575512166</v>
+        <v>411.0273947657205</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>305.5</v>
+        <v>63.8</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,13 +3255,13 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>48.30651527988162</v>
+        <v>56.501300198583</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>18.14262281634702</v>
+        <v>19.18367915910861</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.5320092646604917</v>
+        <v>0.5607948968848361</v>
       </c>
       <c r="K53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>1.174972219069714</v>
+        <v>1.367343591826066</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>6202</v>
+        <v>6187</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>盛群</t>
+          <t>萬潤</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>411.0273947657205</v>
+        <v>409.9965084454129</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>63.8</v>
+        <v>1155</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,16 +3308,16 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>56.501300198583</v>
+        <v>56.82613965776645</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>19.18367915910861</v>
+        <v>12.88446229178037</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.5607948968848361</v>
+        <v>1.499431686737478</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>1.367343591826066</v>
+        <v>19.5731929603824</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>6187</v>
+        <v>6263</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>萬潤</t>
+          <t>普萊德</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>409.9965084454129</v>
+        <v>404.0866976540456</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>1155</v>
+        <v>162.5</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,13 +3361,13 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>56.82613965776645</v>
+        <v>56.96847749368335</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>12.88446229178037</v>
+        <v>11.33714921829252</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>1.499431686737478</v>
+        <v>0.8962451913728131</v>
       </c>
       <c r="K55" s="2" t="n">
         <v>1</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>19.5731929603824</v>
+        <v>1.92142108334208</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6263</v>
+        <v>6188</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>普萊德</t>
+          <t>廣明</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>404.0866976540456</v>
+        <v>403.4278547744497</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>162.5</v>
+        <v>71.8</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,13 +3414,13 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>56.96847749368335</v>
+        <v>49.04695079496783</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>11.33714921829252</v>
+        <v>23.16872008682516</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.8962451913728131</v>
+        <v>0.513925149603626</v>
       </c>
       <c r="K56" s="2" t="n">
         <v>1</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>1.92142108334208</v>
+        <v>0.8093516288072089</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>6188</v>
+        <v>6229</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>廣明</t>
+          <t>研通</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>403.4278547744497</v>
+        <v>402.677806272285</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>71.8</v>
+        <v>23.6</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,16 +3467,16 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>49.04695079496783</v>
+        <v>45.04371545075377</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>23.16872008682516</v>
+        <v>22.92631561134457</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.513925149603626</v>
+        <v>0.3908261039671643</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="L57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.8093516288072089</v>
+        <v>0.1912289670079899</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>6229</v>
+        <v>6412</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>研通</t>
+          <t>群電</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>402.677806272285</v>
+        <v>398.2499757871184</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>23.6</v>
+        <v>79.8</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,16 +3520,16 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>45.04371545075377</v>
+        <v>44.49473955685955</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>22.92631561134457</v>
+        <v>31.33378639371518</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.3908261039671643</v>
+        <v>0.7684293275770844</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.1912289670079899</v>
+        <v>0.4948823338881287</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>6412</v>
+        <v>6411</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>群電</t>
+          <t>晶焱</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>398.2499757871184</v>
+        <v>387.6601941997589</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>79.8</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,16 +3573,16 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>44.49473955685955</v>
+        <v>44.24483719917447</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>31.33378639371518</v>
+        <v>25.66222258753121</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.7684293275770844</v>
+        <v>0.6592837743963089</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.4948823338881287</v>
+        <v>0.884316941250173</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>6411</v>
+        <v>6205</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>晶焱</t>
+          <t>詮欣</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>387.6601941997589</v>
+        <v>386.4363434485523</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>78.90000000000001</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,16 +3626,16 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>44.24483719917447</v>
+        <v>52.44830213572251</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>25.66222258753121</v>
+        <v>27.01750646564948</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.6592837743963089</v>
+        <v>1.220941103905282</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.884316941250173</v>
+        <v>1.362009795316776</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend, cci_momentum</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>6205</v>
+        <v>6291</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>詮欣</t>
+          <t>沛亨</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>386.4363434485523</v>
+        <v>383.9803410082301</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>64.40000000000001</v>
+        <v>402.5</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,16 +3679,16 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>52.44830213572251</v>
+        <v>50.83529474375462</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>27.01750646564948</v>
+        <v>26.9945194114625</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>1.220941103905282</v>
+        <v>1.314947538295888</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L61" s="2" t="n">
         <v>0</v>
@@ -3697,48 +3697,48 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>1.362009795316776</v>
+        <v>11.63168069391828</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend, cci_momentum</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>6291</v>
+        <v>6288</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>沛亨</t>
+          <t>聯嘉</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>383.9803410082301</v>
+        <v>376.0370350697791</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>402.5</v>
+        <v>20.95</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2025-08-04</t>
         </is>
       </c>
       <c r="G62" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>50.83529474375462</v>
+        <v>49.86180348361445</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>26.9945194114625</v>
+        <v>25.01571076609033</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>1.314947538295888</v>
+        <v>0.6831032524092705</v>
       </c>
       <c r="K62" s="2" t="n">
         <v>2</v>
@@ -3750,51 +3750,51 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>11.63168069391828</v>
+        <v>0.0328636758179331</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend</t>
+          <t>ema60_gt_ema120, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6288</v>
+        <v>6462</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>聯嘉</t>
+          <t>神盾</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>376.0370350697791</v>
+        <v>365.3363872554083</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>20.95</v>
+        <v>101.5</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2025-08-04</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G63" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>49.86180348361445</v>
+        <v>48.83752174379585</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>25.01571076609033</v>
+        <v>19.82579509871645</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.6831032524092705</v>
+        <v>0.9497624670529246</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.0328636758179331</v>
+        <v>1.526008235081833</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>6462</v>
+        <v>6456</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>神盾</t>
+          <t>GIS-KY</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>365.3363872554083</v>
+        <v>362.3860762301923</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>101.5</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>48.83752174379585</v>
+        <v>56.05515713935561</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>19.82579509871645</v>
+        <v>19.32739911271666</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.9497624670529246</v>
+        <v>1.139688656056166</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>1.526008235081833</v>
+        <v>1.639194036114024</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>6456</v>
+        <v>6449</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>GIS-KY</t>
+          <t>鈺邦</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>362.3860762301923</v>
+        <v>361.4989807046847</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>68.59999999999999</v>
+        <v>244</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,13 +3891,13 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>56.05515713935561</v>
+        <v>45.98355325648917</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>19.32739911271666</v>
+        <v>30.15602473047489</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>1.139688656056166</v>
+        <v>0.6695199917702532</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0</v>
@@ -3909,31 +3909,31 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>1.639194036114024</v>
+        <v>5.878811941223972</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>6449</v>
+        <v>6259</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>鈺邦</t>
+          <t>百徽</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>361.4989807046847</v>
+        <v>356.1768816733438</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>244</v>
+        <v>31.05</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,16 +3944,16 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>45.98355325648917</v>
+        <v>47.78264511054932</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>30.15602473047489</v>
+        <v>13.57829882176248</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.6695199917702532</v>
+        <v>0.6195123861824808</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>5.878811941223972</v>
+        <v>0.0219779374815631</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>6259</v>
+        <v>6278</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>百徽</t>
+          <t>台表科</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>356.1768816733438</v>
+        <v>353.0773753029393</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>31.05</v>
+        <v>171</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,16 +3997,16 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>47.78264511054932</v>
+        <v>51.8604162116963</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>13.57829882176248</v>
+        <v>25.87739228619832</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.6195123861824808</v>
+        <v>0.9442734563860232</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.0219779374815631</v>
+        <v>3.997116399991867</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>6278</v>
+        <v>6168</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>台表科</t>
+          <t>宏齊</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>353.0773753029393</v>
+        <v>347.3969716473156</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>171</v>
+        <v>25.1</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,13 +4050,13 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>51.8604162116963</v>
+        <v>50.44767418514044</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>25.87739228619832</v>
+        <v>19.37062813623403</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.9442734563860232</v>
+        <v>0.5861136132162559</v>
       </c>
       <c r="K68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>3.997116399991867</v>
+        <v>0.4227163302748959</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>6168</v>
+        <v>6166</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>宏齊</t>
+          <t>凌華</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>347.3969716473156</v>
+        <v>346.6952599333813</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>25.1</v>
+        <v>137</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,13 +4103,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>50.44767418514044</v>
+        <v>50.67617937453824</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>19.37062813623403</v>
+        <v>15.11095825860515</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.5861136132162559</v>
+        <v>0.3199862675109995</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.4227163302748959</v>
+        <v>0.1930964788840367</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>6166</v>
+        <v>6409</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>凌華</t>
+          <t>旭隼</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>346.6952599333813</v>
+        <v>346.2117053270206</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>137</v>
+        <v>995</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>50.67617937453824</v>
+        <v>50.57219158580681</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>15.11095825860515</v>
+        <v>17.42589871111388</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.3199862675109995</v>
+        <v>0.5012084245440042</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.1930964788840367</v>
+        <v>3.567752617774966</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4184,21 +4184,21 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>6409</v>
+        <v>6220</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>旭隼</t>
+          <t>岳豐</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>346.2117053270206</v>
+        <v>344.6470787378587</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>995</v>
+        <v>26.25</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,16 +4209,16 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>50.57219158580681</v>
+        <v>39.28942026583994</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>17.42589871111388</v>
+        <v>30.43611279353573</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.5012084245440042</v>
+        <v>1.162111687455326</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>3.567752617774966</v>
+        <v>0.1744556803796664</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>6220</v>
+        <v>6257</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>岳豐</t>
+          <t>矽格</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>344.6470787378587</v>
+        <v>337.2219429412219</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>26.25</v>
+        <v>211</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,16 +4262,16 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>39.28942026583994</v>
+        <v>50.13604755115158</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>30.43611279353573</v>
+        <v>18.37721706922756</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>1.162111687455326</v>
+        <v>1.282252148911086</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.1744556803796664</v>
+        <v>1.625712180456511</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>6257</v>
+        <v>6196</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>矽格</t>
+          <t>帆宣</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>337.2219429412219</v>
+        <v>336.699400368821</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>211</v>
+        <v>499</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>50.13604755115158</v>
+        <v>47.06886470898647</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>18.37721706922756</v>
+        <v>16.07179495848317</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>1.282252148911086</v>
+        <v>0.701188068528297</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>1.625712180456511</v>
+        <v>1.382916123357044</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>6196</v>
+        <v>6441</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>帆宣</t>
+          <t>廣錠</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>336.699400368821</v>
+        <v>330.9923333888228</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>499</v>
+        <v>22.6</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>47.06886470898647</v>
+        <v>57.26750771504849</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>16.07179495848317</v>
+        <v>20.11594810745253</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.701188068528297</v>
+        <v>0.8279316398449599</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>1.382916123357044</v>
+        <v>0.4679177984567606</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6441</v>
+        <v>6226</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>廣錠</t>
+          <t>光鼎</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>330.9923333888228</v>
+        <v>325.3962906049626</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>22.6</v>
+        <v>20.3</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,13 +4421,13 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>57.26750771504849</v>
+        <v>48.64551819321513</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>20.11594810745253</v>
+        <v>19.69338597219521</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.8279316398449599</v>
+        <v>0.3800088280479545</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.4679177984567606</v>
+        <v>-0.2151284842289763</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>6226</v>
+        <v>6209</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>光鼎</t>
+          <t>今國光</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>325.3962906049626</v>
+        <v>322.4135920360185</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>20.3</v>
+        <v>75</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,13 +4474,13 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>48.64551819321513</v>
+        <v>52.91149193880289</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>19.69338597219521</v>
+        <v>15.67707408877657</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.3800088280479545</v>
+        <v>0.8157248372425977</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>0</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.2151284842289763</v>
+        <v>1.451361105866187</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4502,21 +4502,21 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>6209</v>
+        <v>6237</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>今國光</t>
+          <t>驊訊</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>322.4135920360185</v>
+        <v>308.2720612732168</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>75</v>
+        <v>35.45</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,16 +4527,16 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>52.91149193880289</v>
+        <v>46.28501556492688</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>15.67707408877657</v>
+        <v>31.71053831319534</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.8157248372425977</v>
+        <v>0.7995857671264857</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>1.451361105866187</v>
+        <v>0.6220469760205694</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>6237</v>
+        <v>6281</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>驊訊</t>
+          <t>全國電</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>308.2720612732168</v>
+        <v>306.6985809157759</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>35.45</v>
+        <v>51.7</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,16 +4580,16 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>46.28501556492688</v>
+        <v>51.5447265202068</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>31.71053831319534</v>
+        <v>16.79364574408527</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.7995857671264857</v>
+        <v>0.6867948120168136</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.6220469760205694</v>
+        <v>-0.0274654798016326</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>6281</v>
+        <v>6270</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>全國電</t>
+          <t>倍微</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>306.6985809157759</v>
+        <v>305.4295275723055</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>51.7</v>
+        <v>31.05</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,16 +4633,16 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>51.5447265202068</v>
+        <v>50.1768874616974</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>16.79364574408527</v>
+        <v>16.42674367695991</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.6867948120168136</v>
+        <v>1.070294451412109</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.0274654798016326</v>
+        <v>0.3477943013376059</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>6270</v>
+        <v>6418</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>倍微</t>
+          <t>詠昇</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>305.4295275723055</v>
+        <v>305.07355929222</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>31.05</v>
+        <v>32.6</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,16 +4686,16 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>50.1768874616974</v>
+        <v>54.90483605851916</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>16.42674367695991</v>
+        <v>18.88888146805149</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>1.070294451412109</v>
+        <v>0.2199092230748287</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.3477943013376059</v>
+        <v>0.3348617830180941</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>6418</v>
+        <v>6417</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>詠昇</t>
+          <t>韋僑</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>305.07355929222</v>
+        <v>302.2479737107025</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>32.6</v>
+        <v>112</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,13 +4739,13 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>54.90483605851916</v>
+        <v>41.48454340582838</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>18.88888146805149</v>
+        <v>22.32084653428731</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.2199092230748287</v>
+        <v>0.3849674377821368</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.3348617830180941</v>
+        <v>0.406421119524385</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>6417</v>
+        <v>6182</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>韋僑</t>
+          <t>合晶</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>302.2479737107025</v>
+        <v>299.647787835128</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,29 +4792,29 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>41.48454340582838</v>
+        <v>45.32002858586456</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>22.32084653428731</v>
+        <v>23.7548624359031</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.3849674377821368</v>
+        <v>1.169842982952302</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L82" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M82" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.406421119524385</v>
+        <v>-1.387585636810626</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>

</xml_diff>